<commit_message>
stabilization and export updated
</commit_message>
<xml_diff>
--- a/sal-updated/rawDataset_SAL.xlsx
+++ b/sal-updated/rawDataset_SAL.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,11 +693,6 @@
       <c r="D9" t="n">
         <v>8</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
@@ -714,6 +709,767 @@
       </c>
       <c r="J9" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>45818.52019158565</v>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>-96.11523113886463</v>
+      </c>
+      <c r="I10" t="n">
+        <v>55.9481351</v>
+      </c>
+      <c r="J10" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>45818.52070096065</v>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1603.65</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>962.1880809905001</v>
+      </c>
+      <c r="I11" t="n">
+        <v>58.53123009999999</v>
+      </c>
+      <c r="J11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>45818.52240875</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>326.07</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>195.639485196275</v>
+      </c>
+      <c r="I12" t="n">
+        <v>57.94245370000001</v>
+      </c>
+      <c r="J12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>45818.52286226852</v>
+      </c>
+      <c r="D13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>326.07</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>195.639485196275</v>
+      </c>
+      <c r="I13" t="n">
+        <v>57.94245370000001</v>
+      </c>
+      <c r="J13" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>45818.52290732639</v>
+      </c>
+      <c r="D14" t="n">
+        <v>13</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>326.07</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>195.639485196275</v>
+      </c>
+      <c r="I14" t="n">
+        <v>57.94245370000001</v>
+      </c>
+      <c r="J14" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>45818.52301774306</v>
+      </c>
+      <c r="D15" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>M.C.</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>195.639485196275</v>
+      </c>
+      <c r="I15" t="n">
+        <v>57.94245370000001</v>
+      </c>
+      <c r="J15" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>45818.52323211805</v>
+      </c>
+      <c r="D16" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>326.07</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>195.639485196275</v>
+      </c>
+      <c r="I16" t="n">
+        <v>57.94245370000001</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>45818.53143945602</v>
+      </c>
+      <c r="D17" t="n">
+        <v>16</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>-83.34669394459019</v>
+      </c>
+      <c r="I17" t="n">
+        <v>56.6182111</v>
+      </c>
+      <c r="J17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>45818.54859282407</v>
+      </c>
+      <c r="D18" t="n">
+        <v>17</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>-96.05763562375152</v>
+      </c>
+      <c r="I18" t="n">
+        <v>55.95491030000001</v>
+      </c>
+      <c r="J18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>45818.54947380787</v>
+      </c>
+      <c r="D19" t="n">
+        <v>18</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>-96.05763562375152</v>
+      </c>
+      <c r="I19" t="n">
+        <v>55.95491030000001</v>
+      </c>
+      <c r="J19" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>45818.55005805555</v>
+      </c>
+      <c r="D20" t="n">
+        <v>19</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>-96.05763562375152</v>
+      </c>
+      <c r="I20" t="n">
+        <v>55.95491030000001</v>
+      </c>
+      <c r="J20" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>45818.55008127315</v>
+      </c>
+      <c r="D21" t="n">
+        <v>20</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>-96.05763562375152</v>
+      </c>
+      <c r="I21" t="n">
+        <v>55.95491030000001</v>
+      </c>
+      <c r="J21" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>45818.5529015625</v>
+      </c>
+      <c r="D22" t="n">
+        <v>21</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>-81.20838528789049</v>
+      </c>
+      <c r="I22" t="n">
+        <v>56.67382360000001</v>
+      </c>
+      <c r="J22" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>45818.55379043982</v>
+      </c>
+      <c r="D23" t="n">
+        <v>22</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>-81.20838528789049</v>
+      </c>
+      <c r="I23" t="n">
+        <v>56.67382360000001</v>
+      </c>
+      <c r="J23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>45818.55381290509</v>
+      </c>
+      <c r="D24" t="n">
+        <v>23</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>-81.20838528789049</v>
+      </c>
+      <c r="I24" t="n">
+        <v>56.67382360000001</v>
+      </c>
+      <c r="J24" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>45818.55792141204</v>
+      </c>
+      <c r="D25" t="n">
+        <v>24</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I25" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J25" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="b">
+        <v>1</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>45818.55829056713</v>
+      </c>
+      <c r="D26" t="n">
+        <v>25</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I26" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J26" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="b">
+        <v>1</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>45818.55831199074</v>
+      </c>
+      <c r="D27" t="n">
+        <v>26</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I27" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J27" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="b">
+        <v>1</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>45818.55882462963</v>
+      </c>
+      <c r="D28" t="n">
+        <v>27</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I28" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J28" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="b">
+        <v>1</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>45818.55884245371</v>
+      </c>
+      <c r="D29" t="n">
+        <v>28</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I29" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J29" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="b">
+        <v>1</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>45818.5595853125</v>
+      </c>
+      <c r="D30" t="n">
+        <v>29</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I30" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J30" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="b">
+        <v>1</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>45818.55960236111</v>
+      </c>
+      <c r="D31" t="n">
+        <v>30</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I31" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J31" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="b">
+        <v>1</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>45818.56010893518</v>
+      </c>
+      <c r="D32" t="n">
+        <v>31</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I32" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="b">
+        <v>1</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>45818.56036958333</v>
+      </c>
+      <c r="D33" t="n">
+        <v>32</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I33" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="b">
+        <v>1</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>45818.56043078704</v>
+      </c>
+      <c r="D34" t="n">
+        <v>33</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I34" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="b">
+        <v>1</v>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>45818.56145732639</v>
+      </c>
+      <c r="D35" t="n">
+        <v>34</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I35" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="b">
+        <v>1</v>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>45818.56151820602</v>
+      </c>
+      <c r="D36" t="n">
+        <v>35</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>N.D.</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>-97.55982770572169</v>
+      </c>
+      <c r="I36" t="n">
+        <v>55.73406969999999</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1232</v>
       </c>
     </row>
   </sheetData>
@@ -727,7 +1483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1041,11 +1797,6 @@
       <c r="C9" t="n">
         <v>8</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
@@ -1054,15 +1805,11 @@
           <t>Manual</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>3232</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>35545454656</t>
-        </is>
+      <c r="G9" t="n">
+        <v>3232</v>
+      </c>
+      <c r="H9" t="n">
+        <v>35545454656</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
@@ -1077,6 +1824,912 @@
         <v>120</v>
       </c>
       <c r="M9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>45818.52019158565</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L10" t="n">
+        <v>120</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>45818.52070096065</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>120</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>45818.52240875</v>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>120</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>45818.52286226852</v>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L13" t="n">
+        <v>120</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>45818.52290732639</v>
+      </c>
+      <c r="C14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L14" t="n">
+        <v>120</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>45818.52301774306</v>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>120</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>45818.52323211805</v>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L16" t="n">
+        <v>120</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>45818.53143945602</v>
+      </c>
+      <c r="C17" t="n">
+        <v>16</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L17" t="n">
+        <v>120</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>45818.54859282407</v>
+      </c>
+      <c r="C18" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L18" t="n">
+        <v>120</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>45818.54947380787</v>
+      </c>
+      <c r="C19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L19" t="n">
+        <v>120</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>45818.55005805555</v>
+      </c>
+      <c r="C20" t="n">
+        <v>19</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L20" t="n">
+        <v>120</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>45818.55008127315</v>
+      </c>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L21" t="n">
+        <v>120</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>45818.5529015625</v>
+      </c>
+      <c r="C22" t="n">
+        <v>21</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>120</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>45818.55379043982</v>
+      </c>
+      <c r="C23" t="n">
+        <v>22</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>120</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>45818.55381290509</v>
+      </c>
+      <c r="C24" t="n">
+        <v>23</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>120</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>45818.55792141204</v>
+      </c>
+      <c r="C25" t="n">
+        <v>24</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L25" t="n">
+        <v>120</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>45818.55829056713</v>
+      </c>
+      <c r="C26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L26" t="n">
+        <v>120</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>45818.55831199074</v>
+      </c>
+      <c r="C27" t="n">
+        <v>26</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L27" t="n">
+        <v>120</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>45818.55882462963</v>
+      </c>
+      <c r="C28" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L28" t="n">
+        <v>120</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>45818.55884245371</v>
+      </c>
+      <c r="C29" t="n">
+        <v>28</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L29" t="n">
+        <v>120</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>45818.5595853125</v>
+      </c>
+      <c r="C30" t="n">
+        <v>29</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>100</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L30" t="n">
+        <v>120</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>45818.55960236111</v>
+      </c>
+      <c r="C31" t="n">
+        <v>30</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>100</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L31" t="n">
+        <v>120</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>45818.56010893518</v>
+      </c>
+      <c r="C32" t="n">
+        <v>31</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>1212</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L32" t="n">
+        <v>120</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>45818.56036958333</v>
+      </c>
+      <c r="C33" t="n">
+        <v>32</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>1212</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L33" t="n">
+        <v>120</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>45818.56043078704</v>
+      </c>
+      <c r="C34" t="n">
+        <v>33</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L34" t="n">
+        <v>120</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>45818.56145732639</v>
+      </c>
+      <c r="C35" t="n">
+        <v>34</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L35" t="n">
+        <v>120</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>45818.56151820602</v>
+      </c>
+      <c r="C36" t="n">
+        <v>35</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>1232</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L36" t="n">
+        <v>120</v>
+      </c>
+      <c r="M36" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1093,7 +2746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1344,17 +2997,13 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>45817.56871664818</v>
+        <v>45817.56871664352</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
         <v>8</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>0</v>
       </c>
@@ -1372,6 +3021,739 @@
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>45818.52019158565</v>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G10" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I10" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>45818.52070096065</v>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G11" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H11" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I11" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>45818.52240875</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G12" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H12" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I12" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>45818.52286226852</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G13" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H13" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I13" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>45818.52290732639</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="n">
+        <v>13</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G14" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H14" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I14" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>45818.52301774306</v>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G15" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H15" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I15" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>45818.52323211805</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G16" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H16" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I16" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>45818.53143945602</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="n">
+        <v>16</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G17" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H17" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I17" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>45818.54859282407</v>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="n">
+        <v>17</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G18" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H18" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I18" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>45818.54947380787</v>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G19" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H19" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I19" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>45818.55005805555</v>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="n">
+        <v>19</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G20" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H20" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I20" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>45818.55008127315</v>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G21" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H21" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I21" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>45818.5529015625</v>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>21</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G22" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H22" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I22" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>45818.55379043982</v>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="n">
+        <v>22</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G23" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H23" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I23" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>45818.55381290509</v>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="n">
+        <v>23</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G24" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H24" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I24" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>45818.55792141204</v>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="n">
+        <v>24</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G25" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H25" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I25" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>45818.55829056713</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>25</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G26" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H26" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I26" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>45818.55831199074</v>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="n">
+        <v>26</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G27" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H27" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I27" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>45818.55882462963</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G28" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H28" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I28" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>45818.55884245371</v>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="n">
+        <v>28</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G29" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H29" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I29" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>45818.5595853125</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="n">
+        <v>29</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G30" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H30" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I30" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>45818.55960236111</v>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="n">
+        <v>30</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G31" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H31" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I31" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>45818.56010893518</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="n">
+        <v>31</v>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G32" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H32" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I32" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>45818.56036958333</v>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="n">
+        <v>32</v>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G33" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H33" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I33" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>45818.56043078704</v>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="n">
+        <v>33</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G34" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H34" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I34" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>45818.56145732639</v>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="n">
+        <v>34</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G35" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I35" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>45818.56151821016</v>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="n">
+        <v>35</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>56.80026</v>
+      </c>
+      <c r="G36" t="n">
+        <v>57.29622609999999</v>
+      </c>
+      <c r="H36" t="n">
+        <v>57.97749800000003</v>
+      </c>
+      <c r="I36" t="n">
+        <v>59.50070250000001</v>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>